<commit_message>
fix case in kpi naming
</commit_message>
<xml_diff>
--- a/dataland-framework-toolbox/inputs/eu-taxonomy-financials/eu-taxonomy-financials.xlsx
+++ b/dataland-framework-toolbox/inputs/eu-taxonomy-financials/eu-taxonomy-financials.xlsx
@@ -109,7 +109,7 @@
     <t>General</t>
   </si>
   <si>
-    <t>Fiscal Year Deviation</t>
+    <t>Fiscal year deviation</t>
   </si>
   <si>
     <t>FISCAL_YEAR_DEVIATION</t>
@@ -127,7 +127,7 @@
     <t>Extended</t>
   </si>
   <si>
-    <t>Fiscal Year End</t>
+    <t>Fiscal year end</t>
   </si>
   <si>
     <t>FISCAL_YEAR_END</t>

</xml_diff>